<commit_message>
feat(reports): improve SIR captions and payment bases
</commit_message>
<xml_diff>
--- a/server/src/main/resources/templates/sir-manual-template.xlsx
+++ b/server/src/main/resources/templates/sir-manual-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIR" sheetId="3" r:id="Re3c0bb349e03427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo Attachment" sheetId="2" r:id="R27fe9b35bc654688"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIR" sheetId="3" r:id="R04ea3a10b9d046ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo Attachment" sheetId="2" r:id="R497275bd648e4d6f"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="xs" localSheetId="1">'Photo Attachment'!$A$1:$N$297</x:definedName>
@@ -13,241 +13,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:si>
-    <x:t xml:space="preserve">SITE INSPECTION REPORT</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CONTRACTOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SITE / SITE #</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">DATE</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">LLC"Avega"</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Kyiv region,                                                           
-SP 28-32-8, Borodyanka, Semashka str., 3.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CONTRACTOR'S REPRESENTATIVE</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">M4H QA STAFF</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">-</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SKILLED LABOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">UNSKILLED LABOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MANAGEMENT ON SITE</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">WEATHER CONDITIONS</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">rainy, +10*С</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ONGOING ACTIVITIES</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BLOCK / LOCATION</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">DESCRIPTION OF WORK (PER BOQ ITEM)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PER SCHEDULE?</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">REMARKS</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">indoor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Water supply system installation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">yes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Heating system installation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Electrical system installation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">no</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sewerage system installation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">outdoor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Roof installation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Walls insulation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">OBSERVANCES ON ONGOING ACTIVITIES</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Installation of cold and hot water supply pipes in insulation tubes. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Installation heating system pipes in insulation tubes. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Heating radiators installation with thermostatic valves. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Installation of electrical cables in corrugated pipe. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Junction boxes installation. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Installation of wooden elements of the roof frame. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Installation of insulation mineral wool plates on the wall along axes A and 4. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">IHP equpment installation. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">OBSERVANCES ON HEALTH &amp; SAFETY</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">YES/NO</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">COMMENTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">All workers wear PPE equipment as relevant.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">yes </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">The fire shield / firefighting equipment is present at site.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">The site is appropriately fenced.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Part of fence was dismantled.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">There is lavatories on the site.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">There are safety briefing logs.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Safety information plate is in tact.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Scaffolding equipment have not secuerily base. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">must be made and installed in accordance with clause 7.3 of DBN A.3.2-2-2009. </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">IC drew attantion on the using temporary wiring on the site.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NARRATIVE ASSESSMENT - COMMENTS ON QUALITY</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">WORK</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">COMMENTS ON QUALITY</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">RECTIFICATION REMARKS (NNC / NTC)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">STATUS OF RECTIFICATION</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PURCHASED MATERIALS</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MATERIALS AND EQUIPMENT</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CHARACTERISTICS</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PER DED? (yes/no)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NOTES</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Plaster</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ceresit CT29</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mineral wool plate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Rokwool</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Glue for mineral wool plates</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ceresit CT190</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NARRATIVE ASSESSMENT - COMMENTS ON PROGRESS</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SCHEDULE REVISION REMARKS</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Construction works is carried out slightly behind the Schedule.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">IC recommends increasing the quantity of workers, especially skilled labor to keep up with the Schedule.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NAME</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TITLE</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SIGNATURE</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Pawel Neugebauer</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Report can be filled in electronically, no signature needed.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">END OF REPORT</x:t>
-  </x:si>
   <x:si>
     <x:t xml:space="preserve">Installation wooden elements of the roof frame.</x:t>
   </x:si>
@@ -262,6 +27,9 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Installation of cold water pipes. </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Heating system installation.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Installation electrical cables in corrugated pipe.</x:t>
@@ -1679,7 +1447,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rffed66b6cc8548c7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R94c6226926fb4846"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1711,7 +1479,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R866dd230cb9b48c0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9772b78b1be34b1e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1743,7 +1511,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc9c12398739a49a5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Red130e29d337429f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1775,7 +1543,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rac5102600ad54037"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9bf9e29be6cd4351"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1807,7 +1575,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8080368c06a8463f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rfe9d7630e9914033"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1839,7 +1607,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf94f8061cad14269"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3a57573ca853489b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1871,7 +1639,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6e2368b791174de4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R33c361880d534ac2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1903,7 +1671,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8ec4c57f40004311"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra31c501d730e4ef1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1935,7 +1703,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R43171ab29a9d4ed3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9d1e16f6af0c4d00"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1967,7 +1735,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb9be78071b5f4603"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R50ef838fa22149df"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1999,7 +1767,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re24c37e4d7c54b37"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb3a3efdf42bb471e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2031,7 +1799,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0a147b48466b4add"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R13c75624d759474f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2063,7 +1831,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc11efe6315f644e4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re1e8094e27c54dbb"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2095,7 +1863,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R82de77027cd64bfe"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf5c0ac16669e4e1c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2127,7 +1895,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R329b765902944cae"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra2d4f74b8e1447df"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2159,7 +1927,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbe7a7e2128d141c0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ref31d065fec541e6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2191,7 +1959,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb1c90d7c129b4dfd"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re6b76caa01c6428b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2223,7 +1991,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rff27894e77f74033"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R084a60e904e242e7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2255,7 +2023,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0722544ff51044e8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd677c42f830d47fd"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2287,7 +2055,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb236b944f4d24ec3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R09bc3b9f58854d70"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2314,7 +2082,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R44f807ca92344d9f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R70110c2ca4164fef"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2341,7 +2109,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R71874f476eb44623"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4d3c464802c44ab4"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2368,7 +2136,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R338bf27def5b4ecf"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rfd3a4659de7a4a82"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2395,7 +2163,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2b308b9121404f13"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0472b920ca6c464e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2422,7 +2190,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R514948a16aa24526"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb7b7fe03877b4629"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2449,7 +2217,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rde50e39f56fc438e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5ad94770d2eb46f6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2698,6 +2466,7 @@
       <x:c r="J1" s="45"/>
       <x:c r="K1" s="45"/>
       <x:c r="L1" s="46"/>
+      <x:c r="M1"/>
     </x:row>
     <x:row r="2" ht="16.950000762939453" customHeight="1">
       <x:c r="A2" s="47"/>
@@ -2712,10 +2481,11 @@
       <x:c r="J2" s="48"/>
       <x:c r="K2" s="48"/>
       <x:c r="L2" s="49"/>
+      <x:c r="M2"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="69" t="s">
-        <x:v>0</x:v>
+      <x:c r="A3" s="69" t="str">
+        <x:v>SITE INSPECTION REPORT</x:v>
       </x:c>
       <x:c r="B3" s="70"/>
       <x:c r="C3" s="70"/>
@@ -2728,22 +2498,23 @@
       <x:c r="J3" s="71"/>
       <x:c r="K3" s="71"/>
       <x:c r="L3" s="72"/>
+      <x:c r="M3"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="87" t="s">
-        <x:v>1</x:v>
+      <x:c r="A4" s="87" t="str">
+        <x:v>CONTRACTOR</x:v>
       </x:c>
       <x:c r="B4" s="79"/>
       <x:c r="C4" s="79"/>
       <x:c r="D4" s="79"/>
-      <x:c r="E4" s="79" t="s">
-        <x:v>2</x:v>
+      <x:c r="E4" s="79" t="str">
+        <x:v>SITE / SITE #</x:v>
       </x:c>
       <x:c r="F4" s="79"/>
       <x:c r="G4" s="79"/>
       <x:c r="H4" s="79"/>
-      <x:c r="I4" s="73" t="s">
-        <x:v>3</x:v>
+      <x:c r="I4" s="73" t="str">
+        <x:v>DATE</x:v>
       </x:c>
       <x:c r="J4" s="74"/>
       <x:c r="K4" s="74"/>
@@ -2751,34 +2522,36 @@
       <x:c r="M4" s="13"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="88" t="s">
-        <x:v>4</x:v>
+      <x:c r="A5" s="88" t="str">
+        <x:v>LLC"Avega"</x:v>
       </x:c>
       <x:c r="B5" s="77"/>
       <x:c r="C5" s="77"/>
       <x:c r="D5" s="77"/>
-      <x:c r="E5" s="77" t="s">
-        <x:v>5</x:v>
+      <x:c r="E5" s="77" t="str">
+        <x:v>Kyiv region,                                                           
+SP 28-32-8, Borodyanka, Semashka str., 3.</x:v>
       </x:c>
       <x:c r="F5" s="77"/>
       <x:c r="G5" s="77"/>
       <x:c r="H5" s="77"/>
-      <x:c r="I5" s="76">
+      <x:c r="I5" s="76" t="n">
         <x:v>45965</x:v>
       </x:c>
       <x:c r="J5" s="77"/>
       <x:c r="K5" s="77"/>
       <x:c r="L5" s="78"/>
+      <x:c r="M5"/>
     </x:row>
     <x:row r="6" ht="15" customHeight="1">
-      <x:c r="A6" s="63" t="s">
-        <x:v>6</x:v>
+      <x:c r="A6" s="63" t="str">
+        <x:v>CONTRACTOR'S REPRESENTATIVE</x:v>
       </x:c>
       <x:c r="B6" s="64"/>
       <x:c r="C6" s="64"/>
       <x:c r="D6" s="65"/>
-      <x:c r="E6" s="66" t="s">
-        <x:v>7</x:v>
+      <x:c r="E6" s="66" t="str">
+        <x:v>UNDP QUALITY ASSURANCE STAFF</x:v>
       </x:c>
       <x:c r="F6" s="64"/>
       <x:c r="G6" s="64"/>
@@ -2792,24 +2565,25 @@
       <x:c r="M6" s="13"/>
     </x:row>
     <x:row r="7" ht="15">
-      <x:c r="A7" s="67" t="s">
-        <x:v>8</x:v>
+      <x:c r="A7" s="67" t="str">
+        <x:v>-</x:v>
       </x:c>
       <x:c r="B7" s="68"/>
       <x:c r="C7" s="68"/>
       <x:c r="D7" s="68"/>
-      <x:c r="E7" s="68">
+      <x:c r="E7" s="68" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F7" s="68"/>
       <x:c r="G7" s="68"/>
       <x:c r="H7" s="68"/>
-      <x:c r="I7" s="81">
+      <x:c r="I7" s="81" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J7" s="82"/>
       <x:c r="K7" s="82"/>
       <x:c r="L7" s="83"/>
+      <x:c r="M7"/>
     </x:row>
     <x:row r="8" ht="15">
       <x:c r="A8" s="84"/>
@@ -2824,54 +2598,57 @@
       <x:c r="J8" s="85"/>
       <x:c r="K8" s="85"/>
       <x:c r="L8" s="86"/>
+      <x:c r="M8"/>
     </x:row>
     <x:row r="9" ht="15" customHeight="1">
-      <x:c r="A9" s="59" t="s">
-        <x:v>9</x:v>
+      <x:c r="A9" s="59" t="str">
+        <x:v>SKILLED LABOR</x:v>
       </x:c>
       <x:c r="B9" s="60"/>
-      <x:c r="C9" s="57" t="s">
-        <x:v>10</x:v>
+      <x:c r="C9" s="57" t="str">
+        <x:v>UNSKILLED LABOR</x:v>
       </x:c>
       <x:c r="D9" s="58"/>
-      <x:c r="E9" s="50" t="s">
-        <x:v>11</x:v>
+      <x:c r="E9" s="50" t="str">
+        <x:v>MANAGEMENT ON SITE</x:v>
       </x:c>
       <x:c r="F9" s="50"/>
       <x:c r="G9" s="50"/>
       <x:c r="H9" s="50"/>
-      <x:c r="I9" s="50" t="s">
-        <x:v>12</x:v>
+      <x:c r="I9" s="50" t="str">
+        <x:v>WEATHER CONDITIONS</x:v>
       </x:c>
       <x:c r="J9" s="50"/>
       <x:c r="K9" s="50"/>
       <x:c r="L9" s="51"/>
+      <x:c r="M9"/>
     </x:row>
     <x:row r="10" ht="15">
-      <x:c r="A10" s="61">
+      <x:c r="A10" s="61" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B10" s="62"/>
-      <x:c r="C10" s="56">
+      <x:c r="C10" s="56" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D10" s="53"/>
-      <x:c r="E10" s="52">
+      <x:c r="E10" s="52" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F10" s="53"/>
       <x:c r="G10" s="53"/>
       <x:c r="H10" s="53"/>
-      <x:c r="I10" s="54" t="s">
-        <x:v>13</x:v>
+      <x:c r="I10" s="54" t="str">
+        <x:v>rainy, +10*С</x:v>
       </x:c>
       <x:c r="J10" s="54"/>
       <x:c r="K10" s="54"/>
       <x:c r="L10" s="55"/>
+      <x:c r="M10"/>
     </x:row>
     <x:row r="11" ht="15" customHeight="1">
-      <x:c r="A11" s="89" t="s">
-        <x:v>14</x:v>
+      <x:c r="A11" s="89" t="str">
+        <x:v>ONGOING ACTIVITIES</x:v>
       </x:c>
       <x:c r="B11" s="90"/>
       <x:c r="C11" s="90"/>
@@ -2884,140 +2661,148 @@
       <x:c r="J11" s="90"/>
       <x:c r="K11" s="90"/>
       <x:c r="L11" s="91"/>
+      <x:c r="M11"/>
     </x:row>
     <x:row r="12" ht="31.5" customHeight="1">
-      <x:c r="A12" s="130" t="s">
-        <x:v>15</x:v>
+      <x:c r="A12" s="130" t="str">
+        <x:v>BLOCK / LOCATION</x:v>
       </x:c>
       <x:c r="B12" s="131"/>
-      <x:c r="C12" s="131" t="s">
-        <x:v>16</x:v>
+      <x:c r="C12" s="131" t="str">
+        <x:v>DESCRIPTION OF WORK (PER BOQ ITEM)</x:v>
       </x:c>
       <x:c r="D12" s="131"/>
       <x:c r="E12" s="131"/>
       <x:c r="F12" s="131"/>
       <x:c r="G12" s="131"/>
-      <x:c r="H12" s="131" t="s">
-        <x:v>17</x:v>
+      <x:c r="H12" s="131" t="str">
+        <x:v>PER SCHEDULE?</x:v>
       </x:c>
       <x:c r="I12" s="131"/>
-      <x:c r="J12" s="131" t="s">
-        <x:v>18</x:v>
+      <x:c r="J12" s="131" t="str">
+        <x:v>REMARKS</x:v>
       </x:c>
       <x:c r="K12" s="131"/>
       <x:c r="L12" s="142"/>
+      <x:c r="M12"/>
     </x:row>
     <x:row r="13" ht="17.549999237060547" customHeight="1">
-      <x:c r="A13" s="143" t="s">
-        <x:v>19</x:v>
+      <x:c r="A13" s="143" t="str">
+        <x:v>indoor</x:v>
       </x:c>
       <x:c r="B13" s="144"/>
-      <x:c r="C13" s="22" t="s">
-        <x:v>20</x:v>
+      <x:c r="C13" s="22" t="str">
+        <x:v>Water supply system installation.</x:v>
       </x:c>
       <x:c r="D13" s="23"/>
       <x:c r="E13" s="23"/>
       <x:c r="F13" s="23"/>
       <x:c r="G13" s="24"/>
-      <x:c r="H13" s="20" t="s">
-        <x:v>21</x:v>
+      <x:c r="H13" s="20" t="str">
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="I13" s="21"/>
       <x:c r="J13" s="150"/>
       <x:c r="K13" s="151"/>
       <x:c r="L13" s="152"/>
+      <x:c r="M13"/>
     </x:row>
     <x:row r="14" ht="17.549999237060547" customHeight="1">
       <x:c r="A14" s="145"/>
       <x:c r="B14" s="39"/>
-      <x:c r="C14" s="22" t="s">
-        <x:v>22</x:v>
+      <x:c r="C14" s="22" t="str">
+        <x:v>Heating system installation.</x:v>
       </x:c>
       <x:c r="D14" s="23"/>
       <x:c r="E14" s="23"/>
       <x:c r="F14" s="23"/>
       <x:c r="G14" s="24"/>
-      <x:c r="H14" s="20" t="s">
-        <x:v>21</x:v>
+      <x:c r="H14" s="20" t="str">
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="I14" s="21"/>
       <x:c r="J14" s="150"/>
       <x:c r="K14" s="151"/>
       <x:c r="L14" s="152"/>
+      <x:c r="M14"/>
     </x:row>
     <x:row r="15" ht="17.549999237060547" customHeight="1">
       <x:c r="A15" s="148"/>
       <x:c r="B15" s="149"/>
-      <x:c r="C15" s="22" t="s">
-        <x:v>23</x:v>
+      <x:c r="C15" s="22" t="str">
+        <x:v>Electrical system installation.</x:v>
       </x:c>
       <x:c r="D15" s="23"/>
       <x:c r="E15" s="23"/>
       <x:c r="F15" s="23"/>
       <x:c r="G15" s="24"/>
-      <x:c r="H15" s="20" t="s">
-        <x:v>24</x:v>
+      <x:c r="H15" s="20" t="str">
+        <x:v>no</x:v>
       </x:c>
       <x:c r="I15" s="21"/>
       <x:c r="J15" s="150"/>
       <x:c r="K15" s="151"/>
       <x:c r="L15" s="152"/>
+      <x:c r="M15"/>
     </x:row>
     <x:row r="16" ht="19.799999237060547" customHeight="1">
       <x:c r="A16" s="11"/>
       <x:c r="B16" s="12"/>
-      <x:c r="C16" s="22" t="s">
-        <x:v>25</x:v>
+      <x:c r="C16" s="22" t="str">
+        <x:v>Sewerage system installation.</x:v>
       </x:c>
       <x:c r="D16" s="23"/>
       <x:c r="E16" s="23"/>
       <x:c r="F16" s="23"/>
       <x:c r="G16" s="24"/>
-      <x:c r="H16" s="20" t="s">
-        <x:v>21</x:v>
+      <x:c r="H16" s="20" t="str">
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="I16" s="21"/>
       <x:c r="J16" s="150"/>
       <x:c r="K16" s="151"/>
       <x:c r="L16" s="152"/>
+      <x:c r="M16"/>
     </x:row>
     <x:row r="17" ht="17.549999237060547" customHeight="1">
-      <x:c r="A17" s="146" t="s">
-        <x:v>26</x:v>
+      <x:c r="A17" s="146" t="str">
+        <x:v>outdoor</x:v>
       </x:c>
       <x:c r="B17" s="147"/>
-      <x:c r="C17" s="22" t="s">
-        <x:v>27</x:v>
+      <x:c r="C17" s="22" t="str">
+        <x:v>Roof installation.</x:v>
       </x:c>
       <x:c r="D17" s="23"/>
       <x:c r="E17" s="23"/>
       <x:c r="F17" s="23"/>
       <x:c r="G17" s="24"/>
-      <x:c r="H17" s="20" t="s">
-        <x:v>24</x:v>
+      <x:c r="H17" s="20" t="str">
+        <x:v>no</x:v>
       </x:c>
       <x:c r="I17" s="21"/>
       <x:c r="J17" s="150"/>
       <x:c r="K17" s="151"/>
       <x:c r="L17" s="152"/>
+      <x:c r="M17"/>
     </x:row>
     <x:row r="18" ht="17.549999237060547" customHeight="1">
       <x:c r="A18" s="11"/>
       <x:c r="B18" s="12"/>
-      <x:c r="C18" s="22" t="s">
-        <x:v>28</x:v>
+      <x:c r="C18" s="22" t="str">
+        <x:v>Walls insulation.</x:v>
       </x:c>
       <x:c r="D18" s="23"/>
       <x:c r="E18" s="23"/>
       <x:c r="F18" s="23"/>
       <x:c r="G18" s="24"/>
-      <x:c r="H18" s="20" t="s">
-        <x:v>24</x:v>
+      <x:c r="H18" s="20" t="str">
+        <x:v>no</x:v>
       </x:c>
       <x:c r="I18" s="21"/>
       <x:c r="J18" s="150"/>
       <x:c r="K18" s="151"/>
       <x:c r="L18" s="152"/>
+      <x:c r="M18"/>
     </x:row>
     <x:row r="19" ht="17.549999237060547" customHeight="1">
       <x:c r="A19" s="143"/>
@@ -3032,6 +2817,7 @@
       <x:c r="J19" s="150"/>
       <x:c r="K19" s="151"/>
       <x:c r="L19" s="152"/>
+      <x:c r="M19"/>
     </x:row>
     <x:row r="20" ht="17.549999237060547" customHeight="1">
       <x:c r="A20" s="163"/>
@@ -3046,10 +2832,11 @@
       <x:c r="J20" s="132"/>
       <x:c r="K20" s="133"/>
       <x:c r="L20" s="134"/>
+      <x:c r="M20"/>
     </x:row>
     <x:row r="21" ht="31.5" customHeight="1">
-      <x:c r="A21" s="96" t="s">
-        <x:v>29</x:v>
+      <x:c r="A21" s="96" t="str">
+        <x:v>OBSERVANCES ON ONGOING ACTIVITIES</x:v>
       </x:c>
       <x:c r="B21" s="97"/>
       <x:c r="C21" s="97"/>
@@ -3062,10 +2849,11 @@
       <x:c r="J21" s="97"/>
       <x:c r="K21" s="97"/>
       <x:c r="L21" s="98"/>
+      <x:c r="M21"/>
     </x:row>
     <x:row r="22" ht="17.549999237060547" customHeight="1">
-      <x:c r="A22" s="36" t="s">
-        <x:v>30</x:v>
+      <x:c r="A22" s="36" t="str">
+        <x:v>Installation of cold and hot water supply pipes in insulation tubes. </x:v>
       </x:c>
       <x:c r="B22" s="37"/>
       <x:c r="C22" s="37"/>
@@ -3078,10 +2866,11 @@
       <x:c r="J22" s="37"/>
       <x:c r="K22" s="37"/>
       <x:c r="L22" s="38"/>
+      <x:c r="M22"/>
     </x:row>
     <x:row r="23" ht="16.200000762939453" customHeight="1">
-      <x:c r="A23" s="30" t="s">
-        <x:v>31</x:v>
+      <x:c r="A23" s="30" t="str">
+        <x:v>Installation heating system pipes in insulation tubes. </x:v>
       </x:c>
       <x:c r="B23" s="31"/>
       <x:c r="C23" s="31"/>
@@ -3094,10 +2883,11 @@
       <x:c r="J23" s="31"/>
       <x:c r="K23" s="31"/>
       <x:c r="L23" s="32"/>
+      <x:c r="M23"/>
     </x:row>
     <x:row r="24" ht="16.200000762939453" customHeight="1">
-      <x:c r="A24" s="25" t="s">
-        <x:v>32</x:v>
+      <x:c r="A24" s="25" t="str">
+        <x:v>Heating radiators installation with thermostatic valves. </x:v>
       </x:c>
       <x:c r="B24" s="26"/>
       <x:c r="C24" s="26"/>
@@ -3110,10 +2900,11 @@
       <x:c r="J24" s="26"/>
       <x:c r="K24" s="26"/>
       <x:c r="L24" s="27"/>
+      <x:c r="M24"/>
     </x:row>
     <x:row r="25" ht="16.200000762939453" customHeight="1">
-      <x:c r="A25" s="25" t="s">
-        <x:v>33</x:v>
+      <x:c r="A25" s="25" t="str">
+        <x:v>Installation of electrical cables in corrugated pipe. </x:v>
       </x:c>
       <x:c r="B25" s="26"/>
       <x:c r="C25" s="26"/>
@@ -3126,10 +2917,11 @@
       <x:c r="J25" s="26"/>
       <x:c r="K25" s="26"/>
       <x:c r="L25" s="27"/>
+      <x:c r="M25"/>
     </x:row>
     <x:row r="26" ht="16.200000762939453" customHeight="1">
-      <x:c r="A26" s="25" t="s">
-        <x:v>34</x:v>
+      <x:c r="A26" s="25" t="str">
+        <x:v>Junction boxes installation. </x:v>
       </x:c>
       <x:c r="B26" s="26"/>
       <x:c r="C26" s="26"/>
@@ -3142,10 +2934,11 @@
       <x:c r="J26" s="26"/>
       <x:c r="K26" s="26"/>
       <x:c r="L26" s="27"/>
+      <x:c r="M26"/>
     </x:row>
     <x:row r="27" ht="16.200000762939453" customHeight="1">
-      <x:c r="A27" s="25" t="s">
-        <x:v>35</x:v>
+      <x:c r="A27" s="25" t="str">
+        <x:v>Installation of wooden elements of the roof frame. </x:v>
       </x:c>
       <x:c r="B27" s="26"/>
       <x:c r="C27" s="26"/>
@@ -3158,10 +2951,11 @@
       <x:c r="J27" s="26"/>
       <x:c r="K27" s="26"/>
       <x:c r="L27" s="27"/>
+      <x:c r="M27"/>
     </x:row>
     <x:row r="28" ht="16.200000762939453" customHeight="1">
-      <x:c r="A28" s="25" t="s">
-        <x:v>36</x:v>
+      <x:c r="A28" s="25" t="str">
+        <x:v>Installation of insulation mineral wool plates on the wall along axes A and 4. </x:v>
       </x:c>
       <x:c r="B28" s="26"/>
       <x:c r="C28" s="26"/>
@@ -3174,10 +2968,11 @@
       <x:c r="J28" s="26"/>
       <x:c r="K28" s="26"/>
       <x:c r="L28" s="27"/>
+      <x:c r="M28"/>
     </x:row>
     <x:row r="29" ht="16.200000762939453" customHeight="1">
-      <x:c r="A29" s="25" t="s">
-        <x:v>37</x:v>
+      <x:c r="A29" s="25" t="str">
+        <x:v>IHP equpment installation. </x:v>
       </x:c>
       <x:c r="B29" s="26"/>
       <x:c r="C29" s="26"/>
@@ -3190,6 +2985,7 @@
       <x:c r="J29" s="26"/>
       <x:c r="K29" s="26"/>
       <x:c r="L29" s="27"/>
+      <x:c r="M29"/>
     </x:row>
     <x:row r="30" ht="16.200000762939453" customHeight="1">
       <x:c r="A30" s="33"/>
@@ -3204,10 +3000,11 @@
       <x:c r="J30" s="34"/>
       <x:c r="K30" s="34"/>
       <x:c r="L30" s="35"/>
+      <x:c r="M30"/>
     </x:row>
     <x:row r="31" ht="17.25" customHeight="1">
-      <x:c r="A31" s="96" t="s">
-        <x:v>38</x:v>
+      <x:c r="A31" s="96" t="str">
+        <x:v>OBSERVANCES ON HEALTH &amp; SAFETY</x:v>
       </x:c>
       <x:c r="B31" s="97"/>
       <x:c r="C31" s="97"/>
@@ -3220,6 +3017,7 @@
       <x:c r="J31" s="97"/>
       <x:c r="K31" s="97"/>
       <x:c r="L31" s="98"/>
+      <x:c r="M31"/>
     </x:row>
     <x:row r="32" ht="17.25" customHeight="1">
       <x:c r="A32" s="18"/>
@@ -3229,19 +3027,20 @@
       <x:c r="E32" s="19"/>
       <x:c r="F32" s="19"/>
       <x:c r="G32" s="19"/>
-      <x:c r="H32" s="171" t="s">
-        <x:v>39</x:v>
+      <x:c r="H32" s="171" t="str">
+        <x:v>YES/NO</x:v>
       </x:c>
       <x:c r="I32" s="172"/>
-      <x:c r="J32" s="173" t="s">
-        <x:v>40</x:v>
+      <x:c r="J32" s="173" t="str">
+        <x:v>COMMENTS</x:v>
       </x:c>
       <x:c r="K32" s="173"/>
       <x:c r="L32" s="174"/>
+      <x:c r="M32"/>
     </x:row>
     <x:row r="33" ht="17.25" customHeight="1">
-      <x:c r="A33" s="155" t="s">
-        <x:v>41</x:v>
+      <x:c r="A33" s="155" t="str">
+        <x:v>All workers wear PPE equipment as relevant.</x:v>
       </x:c>
       <x:c r="B33" s="156"/>
       <x:c r="C33" s="156"/>
@@ -3249,17 +3048,18 @@
       <x:c r="E33" s="156"/>
       <x:c r="F33" s="156"/>
       <x:c r="G33" s="157"/>
-      <x:c r="H33" s="208" t="s">
-        <x:v>42</x:v>
+      <x:c r="H33" s="208" t="str">
+        <x:v>yes </x:v>
       </x:c>
       <x:c r="I33" s="158"/>
       <x:c r="J33" s="169"/>
       <x:c r="K33" s="169"/>
       <x:c r="L33" s="170"/>
+      <x:c r="M33"/>
     </x:row>
     <x:row r="34" ht="17.25" customHeight="1">
-      <x:c r="A34" s="159" t="s">
-        <x:v>43</x:v>
+      <x:c r="A34" s="159" t="str">
+        <x:v>The fire shield / firefighting equipment is present at site.</x:v>
       </x:c>
       <x:c r="B34" s="160"/>
       <x:c r="C34" s="160"/>
@@ -3267,17 +3067,18 @@
       <x:c r="E34" s="160"/>
       <x:c r="F34" s="160"/>
       <x:c r="G34" s="161"/>
-      <x:c r="H34" s="209" t="s">
-        <x:v>21</x:v>
+      <x:c r="H34" s="209" t="str">
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="I34" s="162"/>
       <x:c r="J34" s="169"/>
       <x:c r="K34" s="169"/>
       <x:c r="L34" s="170"/>
+      <x:c r="M34"/>
     </x:row>
     <x:row r="35" ht="17.25" customHeight="1">
-      <x:c r="A35" s="159" t="s">
-        <x:v>44</x:v>
+      <x:c r="A35" s="159" t="str">
+        <x:v>The site is appropriately fenced.</x:v>
       </x:c>
       <x:c r="B35" s="160"/>
       <x:c r="C35" s="160"/>
@@ -3285,19 +3086,20 @@
       <x:c r="E35" s="160"/>
       <x:c r="F35" s="160"/>
       <x:c r="G35" s="161"/>
-      <x:c r="H35" s="209" t="s">
-        <x:v>24</x:v>
+      <x:c r="H35" s="209" t="str">
+        <x:v>no</x:v>
       </x:c>
       <x:c r="I35" s="162"/>
-      <x:c r="J35" s="210" t="s">
-        <x:v>45</x:v>
+      <x:c r="J35" s="210" t="str">
+        <x:v>Part of fence was dismantled.</x:v>
       </x:c>
       <x:c r="K35" s="169"/>
       <x:c r="L35" s="170"/>
+      <x:c r="M35"/>
     </x:row>
     <x:row r="36" ht="17.25" customHeight="1">
-      <x:c r="A36" s="159" t="s">
-        <x:v>46</x:v>
+      <x:c r="A36" s="159" t="str">
+        <x:v>There is lavatories on the site.</x:v>
       </x:c>
       <x:c r="B36" s="160"/>
       <x:c r="C36" s="160"/>
@@ -3305,17 +3107,18 @@
       <x:c r="E36" s="160"/>
       <x:c r="F36" s="160"/>
       <x:c r="G36" s="161"/>
-      <x:c r="H36" s="209" t="s">
-        <x:v>21</x:v>
+      <x:c r="H36" s="209" t="str">
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="I36" s="162"/>
       <x:c r="J36" s="169"/>
       <x:c r="K36" s="169"/>
       <x:c r="L36" s="170"/>
+      <x:c r="M36"/>
     </x:row>
     <x:row r="37" ht="16.799999237060547" customHeight="1">
-      <x:c r="A37" s="159" t="s">
-        <x:v>47</x:v>
+      <x:c r="A37" s="159" t="str">
+        <x:v>There are safety briefing logs.</x:v>
       </x:c>
       <x:c r="B37" s="160"/>
       <x:c r="C37" s="160"/>
@@ -3323,17 +3126,18 @@
       <x:c r="E37" s="160"/>
       <x:c r="F37" s="160"/>
       <x:c r="G37" s="161"/>
-      <x:c r="H37" s="209" t="s">
-        <x:v>21</x:v>
+      <x:c r="H37" s="209" t="str">
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="I37" s="162"/>
       <x:c r="J37" s="169"/>
       <x:c r="K37" s="169"/>
       <x:c r="L37" s="170"/>
+      <x:c r="M37"/>
     </x:row>
     <x:row r="38" ht="16.799999237060547" customHeight="1">
-      <x:c r="A38" s="159" t="s">
-        <x:v>48</x:v>
+      <x:c r="A38" s="159" t="str">
+        <x:v>Safety information plate is in tact.</x:v>
       </x:c>
       <x:c r="B38" s="160"/>
       <x:c r="C38" s="160"/>
@@ -3341,17 +3145,18 @@
       <x:c r="E38" s="160"/>
       <x:c r="F38" s="160"/>
       <x:c r="G38" s="161"/>
-      <x:c r="H38" s="209" t="s">
-        <x:v>21</x:v>
+      <x:c r="H38" s="209" t="str">
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="I38" s="162"/>
       <x:c r="J38" s="169"/>
       <x:c r="K38" s="169"/>
       <x:c r="L38" s="170"/>
+      <x:c r="M38"/>
     </x:row>
     <x:row r="39" ht="45.599998474121094" customHeight="1">
-      <x:c r="A39" s="175" t="s">
-        <x:v>49</x:v>
+      <x:c r="A39" s="175" t="str">
+        <x:v>Scaffolding equipment have not secuerily base. </x:v>
       </x:c>
       <x:c r="B39" s="176"/>
       <x:c r="C39" s="176"/>
@@ -3361,15 +3166,16 @@
       <x:c r="G39" s="176"/>
       <x:c r="H39" s="176"/>
       <x:c r="I39" s="176"/>
-      <x:c r="J39" s="179" t="s">
-        <x:v>50</x:v>
+      <x:c r="J39" s="179" t="str">
+        <x:v>must be made and installed in accordance with clause 7.3 of DBN A.3.2-2-2009. </x:v>
       </x:c>
       <x:c r="K39" s="179"/>
       <x:c r="L39" s="180"/>
+      <x:c r="M39"/>
     </x:row>
     <x:row r="40" ht="16.799999237060547" customHeight="1">
-      <x:c r="A40" s="177" t="s">
-        <x:v>51</x:v>
+      <x:c r="A40" s="177" t="str">
+        <x:v>IC drew attantion on the using temporary wiring on the site.</x:v>
       </x:c>
       <x:c r="B40" s="178"/>
       <x:c r="C40" s="178"/>
@@ -3382,6 +3188,7 @@
       <x:c r="J40" s="179"/>
       <x:c r="K40" s="179"/>
       <x:c r="L40" s="180"/>
+      <x:c r="M40"/>
     </x:row>
     <x:row r="41" ht="16.799999237060547" customHeight="1">
       <x:c r="A41" s="165"/>
@@ -3396,10 +3203,11 @@
       <x:c r="J41" s="16"/>
       <x:c r="K41" s="16"/>
       <x:c r="L41" s="17"/>
+      <x:c r="M41"/>
     </x:row>
     <x:row r="42" ht="18" customHeight="1">
-      <x:c r="A42" s="183" t="s">
-        <x:v>52</x:v>
+      <x:c r="A42" s="183" t="str">
+        <x:v>NARRATIVE ASSESSMENT - COMMENTS ON QUALITY</x:v>
       </x:c>
       <x:c r="B42" s="184"/>
       <x:c r="C42" s="184"/>
@@ -3412,28 +3220,30 @@
       <x:c r="J42" s="184"/>
       <x:c r="K42" s="184"/>
       <x:c r="L42" s="185"/>
+      <x:c r="M42"/>
     </x:row>
     <x:row r="43" ht="31.799999237060547" customHeight="1">
-      <x:c r="A43" s="153" t="s">
-        <x:v>53</x:v>
+      <x:c r="A43" s="153" t="str">
+        <x:v>WORK</x:v>
       </x:c>
       <x:c r="B43" s="154"/>
-      <x:c r="C43" s="154" t="s">
-        <x:v>54</x:v>
+      <x:c r="C43" s="154" t="str">
+        <x:v>COMMENTS ON QUALITY</x:v>
       </x:c>
       <x:c r="D43" s="154"/>
       <x:c r="E43" s="154"/>
       <x:c r="F43" s="154"/>
-      <x:c r="G43" s="154" t="s">
-        <x:v>55</x:v>
+      <x:c r="G43" s="154" t="str">
+        <x:v>RECTIFICATION REMARKS (NNC / NTC)</x:v>
       </x:c>
       <x:c r="H43" s="154"/>
       <x:c r="I43" s="154"/>
-      <x:c r="J43" s="128" t="s">
-        <x:v>56</x:v>
+      <x:c r="J43" s="128" t="str">
+        <x:v>STATUS OF RECTIFICATION</x:v>
       </x:c>
       <x:c r="K43" s="128"/>
       <x:c r="L43" s="129"/>
+      <x:c r="M43"/>
     </x:row>
     <x:row r="44" ht="16.200000762939453" customHeight="1">
       <x:c r="A44" s="168"/>
@@ -3448,6 +3258,7 @@
       <x:c r="J44" s="40"/>
       <x:c r="K44" s="41"/>
       <x:c r="L44" s="42"/>
+      <x:c r="M44"/>
     </x:row>
     <x:row r="45" ht="16.200000762939453" customHeight="1">
       <x:c r="A45" s="167"/>
@@ -3462,6 +3273,7 @@
       <x:c r="J45" s="22"/>
       <x:c r="K45" s="23"/>
       <x:c r="L45" s="43"/>
+      <x:c r="M45"/>
     </x:row>
     <x:row r="46" ht="16.200000762939453" customHeight="1">
       <x:c r="A46" s="167"/>
@@ -3476,6 +3288,7 @@
       <x:c r="J46" s="22"/>
       <x:c r="K46" s="23"/>
       <x:c r="L46" s="43"/>
+      <x:c r="M46"/>
     </x:row>
     <x:row r="47" ht="16.200000762939453" customHeight="1">
       <x:c r="A47" s="167"/>
@@ -3490,6 +3303,7 @@
       <x:c r="J47" s="28"/>
       <x:c r="K47" s="28"/>
       <x:c r="L47" s="29"/>
+      <x:c r="M47"/>
     </x:row>
     <x:row r="48" ht="16.200000762939453" customHeight="1">
       <x:c r="A48" s="167"/>
@@ -3504,6 +3318,7 @@
       <x:c r="J48" s="28"/>
       <x:c r="K48" s="28"/>
       <x:c r="L48" s="29"/>
+      <x:c r="M48"/>
     </x:row>
     <x:row r="49" ht="16.200000762939453" customHeight="1">
       <x:c r="A49" s="167"/>
@@ -3518,6 +3333,7 @@
       <x:c r="J49" s="22"/>
       <x:c r="K49" s="23"/>
       <x:c r="L49" s="43"/>
+      <x:c r="M49"/>
     </x:row>
     <x:row r="50" ht="16.200000762939453" customHeight="1">
       <x:c r="A50" s="53"/>
@@ -3532,10 +3348,11 @@
       <x:c r="J50" s="132"/>
       <x:c r="K50" s="133"/>
       <x:c r="L50" s="134"/>
+      <x:c r="M50"/>
     </x:row>
     <x:row r="51" ht="21" customHeight="1">
-      <x:c r="A51" s="96" t="s">
-        <x:v>57</x:v>
+      <x:c r="A51" s="96" t="str">
+        <x:v>PURCHASED MATERIALS</x:v>
       </x:c>
       <x:c r="B51" s="97"/>
       <x:c r="C51" s="97"/>
@@ -3548,88 +3365,93 @@
       <x:c r="J51" s="97"/>
       <x:c r="K51" s="97"/>
       <x:c r="L51" s="98"/>
+      <x:c r="M51"/>
     </x:row>
     <x:row r="52" ht="29.549999237060547" customHeight="1">
-      <x:c r="A52" s="153" t="s">
-        <x:v>58</x:v>
+      <x:c r="A52" s="153" t="str">
+        <x:v>MATERIALS AND EQUIPMENT</x:v>
       </x:c>
       <x:c r="B52" s="154"/>
-      <x:c r="C52" s="154" t="s">
-        <x:v>59</x:v>
+      <x:c r="C52" s="154" t="str">
+        <x:v>CHARACTERISTICS</x:v>
       </x:c>
       <x:c r="D52" s="154"/>
       <x:c r="E52" s="154"/>
       <x:c r="F52" s="154"/>
-      <x:c r="G52" s="154" t="s">
-        <x:v>60</x:v>
+      <x:c r="G52" s="154" t="str">
+        <x:v>PER DED? (yes/no)</x:v>
       </x:c>
       <x:c r="H52" s="154"/>
       <x:c r="I52" s="154"/>
-      <x:c r="J52" s="128" t="s">
-        <x:v>61</x:v>
+      <x:c r="J52" s="128" t="str">
+        <x:v>NOTES</x:v>
       </x:c>
       <x:c r="K52" s="128"/>
       <x:c r="L52" s="129"/>
+      <x:c r="M52"/>
     </x:row>
     <x:row r="53" ht="16.799999237060547" customHeight="1">
-      <x:c r="A53" s="181" t="s">
-        <x:v>62</x:v>
+      <x:c r="A53" s="181" t="str">
+        <x:v>Plaster</x:v>
       </x:c>
       <x:c r="B53" s="182"/>
-      <x:c r="C53" s="182" t="s">
-        <x:v>63</x:v>
+      <x:c r="C53" s="182" t="str">
+        <x:v>Ceresit CT29</x:v>
       </x:c>
       <x:c r="D53" s="182"/>
       <x:c r="E53" s="182"/>
       <x:c r="F53" s="182"/>
-      <x:c r="G53" s="168" t="s">
-        <x:v>21</x:v>
+      <x:c r="G53" s="168" t="str">
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="H53" s="168"/>
       <x:c r="I53" s="168"/>
       <x:c r="J53" s="40"/>
       <x:c r="K53" s="41"/>
       <x:c r="L53" s="42"/>
+      <x:c r="M53"/>
     </x:row>
     <x:row r="54" ht="16.799999237060547" customHeight="1">
-      <x:c r="A54" s="88" t="s">
-        <x:v>64</x:v>
+      <x:c r="A54" s="88" t="str">
+        <x:v>Mineral wool plate</x:v>
       </x:c>
       <x:c r="B54" s="77"/>
-      <x:c r="C54" s="77" t="s">
-        <x:v>65</x:v>
+      <x:c r="C54" s="77" t="str">
+        <x:v>Rokwool</x:v>
       </x:c>
       <x:c r="D54" s="77"/>
       <x:c r="E54" s="77"/>
       <x:c r="F54" s="77"/>
-      <x:c r="G54" s="167" t="s">
-        <x:v>24</x:v>
+      <x:c r="G54" s="167" t="str">
+        <x:v>no</x:v>
       </x:c>
       <x:c r="H54" s="167"/>
       <x:c r="I54" s="167"/>
       <x:c r="J54" s="22"/>
       <x:c r="K54" s="23"/>
       <x:c r="L54" s="43"/>
+      <x:c r="M54"/>
     </x:row>
     <x:row r="55" ht="34.20000076293945" customHeight="1">
-      <x:c r="A55" s="88" t="s">
-        <x:v>66</x:v>
+      <x:c r="A55" s="88" t="str">
+        <x:v>Glue for mineral wool plates</x:v>
       </x:c>
       <x:c r="B55" s="77"/>
-      <x:c r="C55" s="167" t="s">
-        <x:v>67</x:v>
+      <x:c r="C55" s="167" t="str">
+        <x:v>Ceresit CT190</x:v>
       </x:c>
       <x:c r="D55" s="167"/>
       <x:c r="E55" s="167"/>
       <x:c r="F55" s="167"/>
-      <x:c r="G55" s="167" t="s">
-        <x:v>21</x:v>
+      <x:c r="G55" s="167" t="str">
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="H55" s="167"/>
       <x:c r="I55" s="167"/>
       <x:c r="J55" s="22"/>
       <x:c r="K55" s="23"/>
       <x:c r="L55" s="43"/>
+      <x:c r="M55"/>
     </x:row>
     <x:row r="56" ht="16.799999237060547" customHeight="1">
       <x:c r="A56" s="186"/>
@@ -3644,6 +3466,7 @@
       <x:c r="J56" s="28"/>
       <x:c r="K56" s="28"/>
       <x:c r="L56" s="29"/>
+      <x:c r="M56"/>
     </x:row>
     <x:row r="57" ht="16.799999237060547" customHeight="1">
       <x:c r="A57" s="186"/>
@@ -3658,6 +3481,7 @@
       <x:c r="J57" s="28"/>
       <x:c r="K57" s="28"/>
       <x:c r="L57" s="29"/>
+      <x:c r="M57"/>
     </x:row>
     <x:row r="58" ht="16.799999237060547" customHeight="1">
       <x:c r="A58" s="186"/>
@@ -3672,6 +3496,7 @@
       <x:c r="J58" s="22"/>
       <x:c r="K58" s="23"/>
       <x:c r="L58" s="43"/>
+      <x:c r="M58"/>
     </x:row>
     <x:row r="59" ht="16.799999237060547" customHeight="1">
       <x:c r="A59" s="187"/>
@@ -3686,10 +3511,11 @@
       <x:c r="J59" s="132"/>
       <x:c r="K59" s="133"/>
       <x:c r="L59" s="134"/>
+      <x:c r="M59"/>
     </x:row>
     <x:row r="60" ht="15" customHeight="1">
-      <x:c r="A60" s="113" t="s">
-        <x:v>68</x:v>
+      <x:c r="A60" s="113" t="str">
+        <x:v>NARRATIVE ASSESSMENT - COMMENTS ON PROGRESS</x:v>
       </x:c>
       <x:c r="B60" s="114"/>
       <x:c r="C60" s="114"/>
@@ -3699,15 +3525,16 @@
       <x:c r="G60" s="114"/>
       <x:c r="H60" s="114"/>
       <x:c r="I60" s="115"/>
-      <x:c r="J60" s="114" t="s">
-        <x:v>69</x:v>
+      <x:c r="J60" s="114" t="str">
+        <x:v>SCHEDULE REVISION REMARKS</x:v>
       </x:c>
       <x:c r="K60" s="114"/>
       <x:c r="L60" s="115"/>
+      <x:c r="M60"/>
     </x:row>
     <x:row r="61" ht="49.79999923706055" customHeight="1">
-      <x:c r="A61" s="116" t="s">
-        <x:v>70</x:v>
+      <x:c r="A61" s="116" t="str">
+        <x:v>Construction works is carried out slightly behind the Schedule.</x:v>
       </x:c>
       <x:c r="B61" s="28"/>
       <x:c r="C61" s="28"/>
@@ -3717,11 +3544,12 @@
       <x:c r="G61" s="28"/>
       <x:c r="H61" s="28"/>
       <x:c r="I61" s="28"/>
-      <x:c r="J61" s="40" t="s">
-        <x:v>71</x:v>
+      <x:c r="J61" s="40" t="str">
+        <x:v>IC recommends increasing the quantity of workers, especially skilled labor to keep up with the Schedule.</x:v>
       </x:c>
       <x:c r="K61" s="41"/>
       <x:c r="L61" s="42"/>
+      <x:c r="M61"/>
     </x:row>
     <x:row r="62" ht="15">
       <x:c r="A62" s="117"/>
@@ -3736,10 +3564,11 @@
       <x:c r="J62" s="22"/>
       <x:c r="K62" s="23"/>
       <x:c r="L62" s="43"/>
+      <x:c r="M62"/>
     </x:row>
     <x:row r="63" ht="16.950000762939453" customHeight="1">
-      <x:c r="A63" s="96" t="s">
-        <x:v>7</x:v>
+      <x:c r="A63" s="96" t="str">
+        <x:v>UNDP QUALITY ASSURANCE STAFF</x:v>
       </x:c>
       <x:c r="B63" s="97"/>
       <x:c r="C63" s="97"/>
@@ -3752,28 +3581,30 @@
       <x:c r="J63" s="97"/>
       <x:c r="K63" s="97"/>
       <x:c r="L63" s="98"/>
+      <x:c r="M63"/>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="99" t="s">
-        <x:v>72</x:v>
+      <x:c r="A64" s="99" t="str">
+        <x:v>NAME</x:v>
       </x:c>
       <x:c r="B64" s="100"/>
       <x:c r="C64" s="100"/>
-      <x:c r="D64" s="103" t="s">
-        <x:v>73</x:v>
+      <x:c r="D64" s="103" t="str">
+        <x:v>TITLE</x:v>
       </x:c>
       <x:c r="E64" s="104"/>
-      <x:c r="F64" s="100" t="s">
-        <x:v>3</x:v>
+      <x:c r="F64" s="100" t="str">
+        <x:v>DATE</x:v>
       </x:c>
       <x:c r="G64" s="104"/>
-      <x:c r="H64" s="107" t="s">
-        <x:v>74</x:v>
+      <x:c r="H64" s="107" t="str">
+        <x:v>SIGNATURE</x:v>
       </x:c>
       <x:c r="I64" s="108"/>
       <x:c r="J64" s="108"/>
       <x:c r="K64" s="108"/>
       <x:c r="L64" s="109"/>
+      <x:c r="M64"/>
     </x:row>
     <x:row r="65" ht="15">
       <x:c r="A65" s="101"/>
@@ -3788,10 +3619,11 @@
       <x:c r="J65" s="111"/>
       <x:c r="K65" s="111"/>
       <x:c r="L65" s="112"/>
+      <x:c r="M65"/>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="118" t="s">
-        <x:v>75</x:v>
+      <x:c r="A66" s="118" t="str">
+        <x:v>Pawel Neugebauer</x:v>
       </x:c>
       <x:c r="B66" s="119"/>
       <x:c r="C66" s="120"/>
@@ -3799,7 +3631,7 @@
         <x:v>TL IC</x:v>
       </x:c>
       <x:c r="E66" s="120"/>
-      <x:c r="F66" s="127">
+      <x:c r="F66" s="127" t="n">
         <x:v>45965</x:v>
       </x:c>
       <x:c r="G66" s="120"/>
@@ -3808,6 +3640,7 @@
       <x:c r="J66" s="136"/>
       <x:c r="K66" s="136"/>
       <x:c r="L66" s="137"/>
+      <x:c r="M66"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="118"/>
@@ -3822,6 +3655,7 @@
       <x:c r="J67" s="138"/>
       <x:c r="K67" s="138"/>
       <x:c r="L67" s="137"/>
+      <x:c r="M67"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="122"/>
@@ -3836,10 +3670,11 @@
       <x:c r="J68" s="140"/>
       <x:c r="K68" s="140"/>
       <x:c r="L68" s="141"/>
+      <x:c r="M68"/>
     </x:row>
     <x:row r="69" ht="16.200000762939453">
-      <x:c r="A69" s="94" t="s">
-        <x:v>76</x:v>
+      <x:c r="A69" s="94" t="str">
+        <x:v>Report can be filled in electronically, no signature needed.</x:v>
       </x:c>
       <x:c r="B69" s="95"/>
       <x:c r="C69" s="95"/>
@@ -3850,10 +3685,11 @@
       <x:c r="H69" s="95"/>
       <x:c r="I69" s="95"/>
       <x:c r="J69" s="95"/>
-      <x:c r="K69" s="92" t="s">
-        <x:v>77</x:v>
+      <x:c r="K69" s="92" t="str">
+        <x:v>END OF REPORT</x:v>
       </x:c>
       <x:c r="L69" s="93"/>
+      <x:c r="M69"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4430,7 +4266,7 @@
       <x:c r="C29" s="5"/>
       <x:c r="D29" s="5"/>
       <x:c r="E29" s="202" t="s">
-        <x:v>78</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F29" s="202"/>
       <x:c r="G29" s="202"/>
@@ -4834,7 +4670,7 @@
     </x:row>
     <x:row r="58">
       <x:c r="B58" s="201" t="s">
-        <x:v>78</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C58" s="202"/>
       <x:c r="D58" s="202"/>
@@ -5260,7 +5096,7 @@
     </x:row>
     <x:row r="90">
       <x:c r="B90" s="201" t="s">
-        <x:v>79</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C90" s="202"/>
       <x:c r="D90" s="202"/>
@@ -5640,7 +5476,7 @@
     <x:row r="117">
       <x:c r="B117" s="4"/>
       <x:c r="C117" s="192" t="s">
-        <x:v>79</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D117" s="192"/>
       <x:c r="E117" s="192"/>
@@ -6049,7 +5885,7 @@
     </x:row>
     <x:row r="148">
       <x:c r="B148" s="191" t="s">
-        <x:v>79</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C148" s="192"/>
       <x:c r="D148" s="192"/>
@@ -6470,7 +6306,7 @@
     </x:row>
     <x:row r="178">
       <x:c r="B178" s="204" t="s">
-        <x:v>80</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C178" s="197"/>
       <x:c r="D178" s="197"/>
@@ -6866,7 +6702,7 @@
     </x:row>
     <x:row r="208">
       <x:c r="B208" s="191" t="s">
-        <x:v>81</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C208" s="192"/>
       <x:c r="D208" s="192"/>
@@ -7263,7 +7099,7 @@
     </x:row>
     <x:row r="237" ht="30" customHeight="1">
       <x:c r="B237" s="194" t="s">
-        <x:v>81</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C237" s="195"/>
       <x:c r="D237" s="195"/>
@@ -7661,7 +7497,7 @@
     </x:row>
     <x:row r="267">
       <x:c r="B267" s="191" t="s">
-        <x:v>82</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C267" s="192"/>
       <x:c r="D267" s="192"/>
@@ -8055,7 +7891,7 @@
     </x:row>
     <x:row r="295" ht="30" customHeight="1">
       <x:c r="B295" s="188" t="s">
-        <x:v>22</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C295" s="197"/>
       <x:c r="D295" s="197"/>
@@ -8467,7 +8303,7 @@
     </x:row>
     <x:row r="326" ht="29.25" customHeight="1">
       <x:c r="B326" s="194" t="s">
-        <x:v>83</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C326" s="199"/>
       <x:c r="D326" s="199"/>
@@ -8847,7 +8683,7 @@
     </x:row>
     <x:row r="353" ht="30" customHeight="1">
       <x:c r="B353" s="188" t="s">
-        <x:v>84</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C353" s="197"/>
       <x:c r="D353" s="197"/>
@@ -9259,7 +9095,7 @@
     </x:row>
     <x:row r="384" ht="29.25" customHeight="1">
       <x:c r="B384" s="194" t="s">
-        <x:v>85</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C384" s="199"/>
       <x:c r="D384" s="199"/>
@@ -9639,7 +9475,7 @@
     </x:row>
     <x:row r="411" ht="30" customHeight="1">
       <x:c r="B411" s="188" t="s">
-        <x:v>86</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C411" s="197"/>
       <x:c r="D411" s="197"/>
@@ -10429,7 +10265,7 @@
     </x:row>
     <x:row r="469" ht="30" customHeight="1">
       <x:c r="B469" s="188" t="s">
-        <x:v>84</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C469" s="197"/>
       <x:c r="D469" s="197"/>
@@ -10827,7 +10663,7 @@
     </x:row>
     <x:row r="499">
       <x:c r="B499" s="191" t="s">
-        <x:v>87</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C499" s="192"/>
       <x:c r="D499" s="192"/>
@@ -11201,7 +11037,7 @@
     </x:row>
     <x:row r="527" ht="30" customHeight="1">
       <x:c r="B527" s="188" t="s">
-        <x:v>88</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C527" s="189"/>
       <x:c r="D527" s="189"/>
@@ -11599,7 +11435,7 @@
     </x:row>
     <x:row r="557">
       <x:c r="B557" s="191" t="s">
-        <x:v>89</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C557" s="192"/>
       <x:c r="D557" s="192"/>
@@ -11973,7 +11809,7 @@
     </x:row>
     <x:row r="585">
       <x:c r="B585" s="188" t="s">
-        <x:v>90</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C585" s="189"/>
       <x:c r="D585" s="189"/>
@@ -12368,7 +12204,7 @@
     </x:row>
     <x:row r="615">
       <x:c r="B615" s="191" t="s">
-        <x:v>91</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C615" s="192"/>
       <x:c r="D615" s="192"/>
@@ -13135,7 +12971,7 @@
     </x:row>
     <x:row r="673">
       <x:c r="B673" s="191" t="s">
-        <x:v>92</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C673" s="192"/>
       <x:c r="D673" s="192"/>
@@ -13509,7 +13345,7 @@
     </x:row>
     <x:row r="701">
       <x:c r="B701" s="188" t="s">
-        <x:v>93</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C701" s="189"/>
       <x:c r="D701" s="189"/>
@@ -13904,7 +13740,7 @@
     </x:row>
     <x:row r="731">
       <x:c r="B731" s="191" t="s">
-        <x:v>94</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C731" s="192"/>
       <x:c r="D731" s="192"/>
@@ -14278,7 +14114,7 @@
     </x:row>
     <x:row r="759">
       <x:c r="B759" s="188" t="s">
-        <x:v>95</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C759" s="189"/>
       <x:c r="D759" s="189"/>
@@ -14673,7 +14509,7 @@
     </x:row>
     <x:row r="789">
       <x:c r="B789" s="191" t="s">
-        <x:v>96</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C789" s="192"/>
       <x:c r="D789" s="192"/>
@@ -15128,6 +14964,6 @@
     <x:mergeCell ref="B789:M789"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdff7c2fec1344a79"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1409d30bc5814cc8"/>
 </x:worksheet>
 </file>
</xml_diff>